<commit_message>
Updated to work with IFC 4.0, IFC version is now a flag. More info @ readme.
</commit_message>
<xml_diff>
--- a/GML2IFC/schema.xlsx
+++ b/GML2IFC/schema.xlsx
@@ -449,7 +449,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -471,7 +470,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
@@ -497,7 +495,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CityGML element/class/function -&gt; IFC class</t>
+          <t>CityGML element/class/function -&gt; IFC class, for IFC 4.3 (default) and IFC4</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -523,7 +521,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -549,14 +546,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
-    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -572,15 +571,25 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>IFC class</t>
+          <t>IFC class (4.3, default)</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>Spatial relation</t>
+          <t>Spatial relation (4.3)</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>IFC class (IFC4, --ifc-version 4)</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Spatial relation (IFC4)</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Note / label</t>
         </is>
@@ -609,6 +618,16 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>IfcBuilding</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>IfcRelAggregates (Site -&gt; Building)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>LOD2 solid preferred, LOD0 footprint fallback (see module docstring)</t>
         </is>
       </c>
@@ -636,6 +655,16 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>IfcWall</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>IfcRelContainedInSpatialStructure (Site -&gt; Element)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
           <t>Mur (wall)</t>
         </is>
       </c>
@@ -663,6 +692,16 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>IfcWall</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>IfcRelContainedInSpatialStructure (Site -&gt; Element)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
           <t>Stödmur (retaining wall)</t>
         </is>
       </c>
@@ -690,6 +729,16 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>IfcCivilElement (ObjectType=Road)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>IfcRelContainedInSpatialStructure (Site -&gt; Element)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
           <t>IfcFacility, aggregated into Site</t>
         </is>
       </c>
@@ -717,6 +766,16 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>IfcCivilElement (ObjectType=Track)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>IfcRelContainedInSpatialStructure (Site -&gt; Element)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
           <t>CityGML 2.0 tran:Track = foot/cycle/horse path, not rail - mapped same as Road</t>
         </is>
       </c>
@@ -744,6 +803,16 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
+          <t>IfcCivilElement (ObjectType=TrafficArea)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>IfcRelContainedInSpatialStructure (Site -&gt; Element)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
           <t>plain IfcElement, contained in Site</t>
         </is>
       </c>
@@ -770,6 +839,16 @@
         </is>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>IfcCivilElement</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>IfcRelContainedInSpatialStructure (Site -&gt; Element)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
         <is>
           <t>original CityGML element tag kept as 'citygmlType' Pset attribute</t>
         </is>
@@ -812,7 +891,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -2558,7 +2636,6 @@
         </is>
       </c>
     </row>
-    <row r="43"/>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
@@ -2754,7 +2831,6 @@
         </is>
       </c>
     </row>
-    <row r="49"/>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>

</xml_diff>